<commit_message>
Task T13 — Registro do parser em parsersBinarios + fidelidade da fixture ao layout real
Registra fatura_itau_cc em parsersBinarios (array ficava vazio em produção mesmo
com parser e roteamento já implementados) e corrige a fixture compartilhada para
trazer o rótulo "Vencimento" acima do serial de vencimento, como no arquivo real,
o que passa a exercitar a regra de parcela antiga (T5) contra a fixture
compartilhada em vez de só contra fixtures construídas em memória.
</commit_message>
<xml_diff>
--- a/src/parsers/__tests__/fixtures/fatura_itau_cc_sintetica.xlsx
+++ b/src/parsers/__tests__/fixtures/fatura_itau_cc_sintetica.xlsx
@@ -17,6 +17,13 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Vencimento</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>

</xml_diff>